<commit_message>
Add login authentication system with Users.xlsx
</commit_message>
<xml_diff>
--- a/docs/assets/Users.xlsx
+++ b/docs/assets/Users.xlsx
@@ -5,15 +5,15 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dell\Documents\Custom Office Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AnnualReportAddin\My Office Add-in\docs\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F1275D4D-61EC-4923-B79B-5B18F229B554}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5B1DBC1-75E5-447D-8D8A-D6417488301A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{426127A8-9F99-448C-B71A-14CD419007A1}"/>
   </bookViews>
   <sheets>
-    <sheet name="User Info" sheetId="1" r:id="rId1"/>
+    <sheet name="Users" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029" concurrentManualCount="12"/>
   <extLst>
@@ -480,6 +480,9 @@
   <we:bindings/>
   <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
   <we:extLst>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
+      <we:containsCustomFunctions/>
+    </a:ext>
     <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{7C84B067-C214-45C3-A712-C9D94CD141B2}">
       <we:customFunctionIdList>
         <we:customFunctionIds>_xldudf_SAP_GETDIMENSIONFILTER</we:customFunctionIds>

</xml_diff>